<commit_message>
Añade hoja Break-Even al modelo financiero
3 escenarios P&L (realista/optimista/target) con proyección 5 años,
tabla de break-even, matriz de sensibilidad presupuesto↔usuarios
y conclusiones de recomendación.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Aristomas_Modelo_Financiero.xlsx
+++ b/Aristomas_Modelo_Financiero.xlsx
@@ -9,6 +9,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supuestos" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Modelo con Churn" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Funnel Marketing" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Break-Even" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1" iterateDelta="0.0001"/>
@@ -17,7 +18,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="7">
+  <numFmts count="8">
     <numFmt numFmtId="164" formatCode="#,##0.00\ \€"/>
     <numFmt numFmtId="165" formatCode="#,##0\ \€"/>
     <numFmt numFmtId="166" formatCode="#,##0\ \€;\(#,##0\ \€\);\-"/>
@@ -25,8 +26,9 @@
     <numFmt numFmtId="168" formatCode="&quot;€&quot;0.00"/>
     <numFmt numFmtId="169" formatCode="0.0%"/>
     <numFmt numFmtId="170" formatCode="&quot;↑&quot;#,##0;&quot;-&quot;#,##0;&quot;=&quot;"/>
+    <numFmt numFmtId="171" formatCode="&quot;€&quot;#,##0;(&quot;€&quot;#,##0);&quot;-&quot;"/>
   </numFmts>
-  <fonts count="29">
+  <fonts count="34">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -209,8 +211,35 @@
       <color rgb="00000000"/>
       <sz val="9"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <color rgb="00666666"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <color rgb="00666666"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00000000"/>
+      <sz val="12"/>
+    </font>
   </fonts>
-  <fills count="27">
+  <fills count="31">
     <fill>
       <patternFill/>
     </fill>
@@ -353,6 +382,30 @@
       <patternFill patternType="solid">
         <fgColor rgb="00FFE0A0"/>
         <bgColor rgb="00FFE0A0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F2F2F2"/>
+        <bgColor rgb="00F2F2F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF0CC"/>
+        <bgColor rgb="00FFF0CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="007A5A0A"/>
+        <bgColor rgb="007A5A0A"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFE0E0"/>
+        <bgColor rgb="00FFE0E0"/>
       </patternFill>
     </fill>
   </fills>
@@ -572,7 +625,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="113">
+  <cellXfs count="169">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -884,6 +937,174 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="28" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="16" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="16" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="17" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="27" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="27" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="24" fillId="19" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="24" fillId="21" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="24" fillId="28" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="24" fillId="19" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="24" fillId="21" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="24" fillId="28" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="24" fillId="19" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="24" fillId="21" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="24" fillId="28" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="22" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="30" fillId="19" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="30" fillId="19" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="24" fillId="25" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="171" fontId="31" fillId="21" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="171" fontId="31" fillId="28" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="24" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="30" fillId="21" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="30" fillId="21" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="29" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="30" fillId="28" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="30" fillId="28" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="16" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="17" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="17" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="30" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="30" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="30" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="21" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="21" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="21" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="28" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="28" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="28" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="27" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="21" fillId="30" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="21" fillId="28" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="21" fillId="21" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="16" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="30" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="30" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="21" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="21" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="28" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="28" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="19" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="19" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -3361,4 +3582,1054 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L62"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="2" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="2" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="13" customWidth="1" min="11" max="11"/>
+    <col width="13" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="34" customHeight="1">
+      <c r="A1" s="113" t="inlineStr">
+        <is>
+          <t>ARISTOMAS · Análisis Break-Even por Escenario de Marketing</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="16" customHeight="1">
+      <c r="A2" s="114" t="inlineStr">
+        <is>
+          <t>Azul=inputs · Negro=fórmulas · Los costes por año son fijos en los 3 escenarios para comparación limpia</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="8" customHeight="1"/>
+    <row r="4" ht="22" customHeight="1">
+      <c r="B4" s="115" t="inlineStr">
+        <is>
+          <t>SUPUESTOS DE PARTIDA</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" s="116" t="inlineStr">
+        <is>
+          <t>Parámetro</t>
+        </is>
+      </c>
+      <c r="C5" s="117" t="inlineStr">
+        <is>
+          <t>Realista</t>
+        </is>
+      </c>
+      <c r="D5" s="117" t="inlineStr">
+        <is>
+          <t>Optimista</t>
+        </is>
+      </c>
+      <c r="E5" s="117" t="inlineStr">
+        <is>
+          <t>Target P&amp;L</t>
+        </is>
+      </c>
+      <c r="F5" s="117" t="inlineStr">
+        <is>
+          <t>Notas</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" s="118" t="inlineStr">
+        <is>
+          <t>Usuarios captados Año 1</t>
+        </is>
+      </c>
+      <c r="C6" s="119" t="n">
+        <v>195</v>
+      </c>
+      <c r="D6" s="120" t="n">
+        <v>515</v>
+      </c>
+      <c r="E6" s="121" t="n">
+        <v>700</v>
+      </c>
+      <c r="F6" s="122" t="inlineStr">
+        <is>
+          <t>Del modelo Funnel Marketing</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" s="118" t="inlineStr">
+        <is>
+          <t>CAC blended estimado (€)</t>
+        </is>
+      </c>
+      <c r="C7" s="123" t="n">
+        <v>83</v>
+      </c>
+      <c r="D7" s="124" t="n">
+        <v>40</v>
+      </c>
+      <c r="E7" s="125" t="n">
+        <v>57</v>
+      </c>
+      <c r="F7" s="122" t="inlineStr">
+        <is>
+          <t>Paid+inf+org / total usuarios</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" s="118" t="inlineStr">
+        <is>
+          <t>ARPU neto (€/usuario/año)</t>
+        </is>
+      </c>
+      <c r="C8" s="123" t="n">
+        <v>83</v>
+      </c>
+      <c r="D8" s="124" t="n">
+        <v>83</v>
+      </c>
+      <c r="E8" s="125" t="n">
+        <v>83</v>
+      </c>
+      <c r="F8" s="122" t="inlineStr">
+        <is>
+          <t>Canónico: 99,99€ ÷ 1,21</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" s="118" t="inlineStr">
+        <is>
+          <t>Churn anual</t>
+        </is>
+      </c>
+      <c r="C9" s="126" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="D9" s="127" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="E9" s="128" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="F9" s="122" t="inlineStr">
+        <is>
+          <t>25% acordado</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" s="118" t="inlineStr">
+        <is>
+          <t>Retención anual</t>
+        </is>
+      </c>
+      <c r="C10" s="126" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="D10" s="127" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="E10" s="128" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="F10" s="122">
+        <f>1−churn</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12" ht="8" customHeight="1"/>
+    <row r="13" ht="24" customHeight="1">
+      <c r="B13" s="129" t="inlineStr">
+        <is>
+          <t>P&amp;L · REALISTA  (195 usuarios Año 1 · CAC paid ~83€)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" s="116" t="inlineStr"/>
+      <c r="C14" s="117" t="inlineStr">
+        <is>
+          <t>Año 1</t>
+        </is>
+      </c>
+      <c r="D14" s="117" t="inlineStr">
+        <is>
+          <t>Año 2</t>
+        </is>
+      </c>
+      <c r="E14" s="117" t="inlineStr">
+        <is>
+          <t>Año 3</t>
+        </is>
+      </c>
+      <c r="F14" s="117" t="inlineStr">
+        <is>
+          <t>Año 4</t>
+        </is>
+      </c>
+      <c r="G14" s="117" t="inlineStr">
+        <is>
+          <t>Año 5</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="19" customHeight="1">
+      <c r="B15" s="118" t="inlineStr">
+        <is>
+          <t>Nuevos usuarios captados</t>
+        </is>
+      </c>
+      <c r="C15" s="96" t="n">
+        <v>195</v>
+      </c>
+      <c r="D15" s="130">
+        <f>C15+100</f>
+        <v/>
+      </c>
+      <c r="E15" s="130">
+        <f>D15+300</f>
+        <v/>
+      </c>
+      <c r="F15" s="130">
+        <f>E15+400</f>
+        <v/>
+      </c>
+      <c r="G15" s="130">
+        <f>F15+350</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16" ht="19" customHeight="1">
+      <c r="B16" s="118" t="inlineStr">
+        <is>
+          <t>Usuarios activos fin de año</t>
+        </is>
+      </c>
+      <c r="C16" s="130">
+        <f>C15</f>
+        <v/>
+      </c>
+      <c r="D16" s="130">
+        <f>ROUND(C15*0.75+D15,0)</f>
+        <v/>
+      </c>
+      <c r="E16" s="130">
+        <f>ROUND(D15*0.75+E15,0)</f>
+        <v/>
+      </c>
+      <c r="F16" s="130">
+        <f>ROUND(E15*0.75+F15,0)</f>
+        <v/>
+      </c>
+      <c r="G16" s="130">
+        <f>ROUND(F15*0.75+G15,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17" ht="19" customHeight="1">
+      <c r="B17" s="118" t="inlineStr">
+        <is>
+          <t>Ingresos (usuarios × 83€)</t>
+        </is>
+      </c>
+      <c r="C17" s="131">
+        <f>C16*83</f>
+        <v/>
+      </c>
+      <c r="D17" s="131">
+        <f>D16*83</f>
+        <v/>
+      </c>
+      <c r="E17" s="131">
+        <f>E16*83</f>
+        <v/>
+      </c>
+      <c r="F17" s="131">
+        <f>F16*83</f>
+        <v/>
+      </c>
+      <c r="G17" s="131">
+        <f>G16*83</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18" ht="19" customHeight="1">
+      <c r="B18" s="118" t="inlineStr">
+        <is>
+          <t>Costes totales</t>
+        </is>
+      </c>
+      <c r="C18" s="132" t="n">
+        <v>120000</v>
+      </c>
+      <c r="D18" s="132" t="n">
+        <v>129000</v>
+      </c>
+      <c r="E18" s="132" t="n">
+        <v>155000</v>
+      </c>
+      <c r="F18" s="132" t="n">
+        <v>175000</v>
+      </c>
+      <c r="G18" s="132" t="n">
+        <v>185000</v>
+      </c>
+    </row>
+    <row r="19" ht="19" customHeight="1">
+      <c r="B19" s="133" t="inlineStr">
+        <is>
+          <t>Resultado anual</t>
+        </is>
+      </c>
+      <c r="C19" s="134">
+        <f>C17-C18</f>
+        <v/>
+      </c>
+      <c r="D19" s="134">
+        <f>D17-D18</f>
+        <v/>
+      </c>
+      <c r="E19" s="134">
+        <f>E17-E18</f>
+        <v/>
+      </c>
+      <c r="F19" s="134">
+        <f>F17-F18</f>
+        <v/>
+      </c>
+      <c r="G19" s="134">
+        <f>G17-G18</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20" ht="19" customHeight="1">
+      <c r="B20" s="133" t="inlineStr">
+        <is>
+          <t>Resultado acumulado</t>
+        </is>
+      </c>
+      <c r="C20" s="135">
+        <f>C19</f>
+        <v/>
+      </c>
+      <c r="D20" s="135">
+        <f>C20+D19</f>
+        <v/>
+      </c>
+      <c r="E20" s="135">
+        <f>D20+E19</f>
+        <v/>
+      </c>
+      <c r="F20" s="135">
+        <f>E20+F19</f>
+        <v/>
+      </c>
+      <c r="G20" s="135">
+        <f>F20+G19</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22" ht="8" customHeight="1"/>
+    <row r="23" ht="24" customHeight="1">
+      <c r="B23" s="136" t="inlineStr">
+        <is>
+          <t>P&amp;L · OPTIMISTA  (515 usuarios Año 1 · CAC paid ~25€)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" s="116" t="inlineStr"/>
+      <c r="C24" s="117" t="inlineStr">
+        <is>
+          <t>Año 1</t>
+        </is>
+      </c>
+      <c r="D24" s="117" t="inlineStr">
+        <is>
+          <t>Año 2</t>
+        </is>
+      </c>
+      <c r="E24" s="117" t="inlineStr">
+        <is>
+          <t>Año 3</t>
+        </is>
+      </c>
+      <c r="F24" s="117" t="inlineStr">
+        <is>
+          <t>Año 4</t>
+        </is>
+      </c>
+      <c r="G24" s="117" t="inlineStr">
+        <is>
+          <t>Año 5</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="19" customHeight="1">
+      <c r="B25" s="118" t="inlineStr">
+        <is>
+          <t>Nuevos usuarios captados</t>
+        </is>
+      </c>
+      <c r="C25" s="96" t="n">
+        <v>515</v>
+      </c>
+      <c r="D25" s="137">
+        <f>C25+100</f>
+        <v/>
+      </c>
+      <c r="E25" s="137">
+        <f>D25+300</f>
+        <v/>
+      </c>
+      <c r="F25" s="137">
+        <f>E25+400</f>
+        <v/>
+      </c>
+      <c r="G25" s="137">
+        <f>F25+350</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26" ht="19" customHeight="1">
+      <c r="B26" s="118" t="inlineStr">
+        <is>
+          <t>Usuarios activos fin de año</t>
+        </is>
+      </c>
+      <c r="C26" s="137">
+        <f>C25</f>
+        <v/>
+      </c>
+      <c r="D26" s="137">
+        <f>ROUND(C25*0.75+D25,0)</f>
+        <v/>
+      </c>
+      <c r="E26" s="137">
+        <f>ROUND(D25*0.75+E25,0)</f>
+        <v/>
+      </c>
+      <c r="F26" s="137">
+        <f>ROUND(E25*0.75+F25,0)</f>
+        <v/>
+      </c>
+      <c r="G26" s="137">
+        <f>ROUND(F25*0.75+G25,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27" ht="19" customHeight="1">
+      <c r="B27" s="118" t="inlineStr">
+        <is>
+          <t>Ingresos (usuarios × 83€)</t>
+        </is>
+      </c>
+      <c r="C27" s="138">
+        <f>C26*83</f>
+        <v/>
+      </c>
+      <c r="D27" s="138">
+        <f>D26*83</f>
+        <v/>
+      </c>
+      <c r="E27" s="138">
+        <f>E26*83</f>
+        <v/>
+      </c>
+      <c r="F27" s="138">
+        <f>F26*83</f>
+        <v/>
+      </c>
+      <c r="G27" s="138">
+        <f>G26*83</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28" ht="19" customHeight="1">
+      <c r="B28" s="118" t="inlineStr">
+        <is>
+          <t>Costes totales</t>
+        </is>
+      </c>
+      <c r="C28" s="132" t="n">
+        <v>120000</v>
+      </c>
+      <c r="D28" s="132" t="n">
+        <v>129000</v>
+      </c>
+      <c r="E28" s="132" t="n">
+        <v>155000</v>
+      </c>
+      <c r="F28" s="132" t="n">
+        <v>175000</v>
+      </c>
+      <c r="G28" s="132" t="n">
+        <v>185000</v>
+      </c>
+    </row>
+    <row r="29" ht="19" customHeight="1">
+      <c r="B29" s="133" t="inlineStr">
+        <is>
+          <t>Resultado anual</t>
+        </is>
+      </c>
+      <c r="C29" s="134">
+        <f>C27-C28</f>
+        <v/>
+      </c>
+      <c r="D29" s="134">
+        <f>D27-D28</f>
+        <v/>
+      </c>
+      <c r="E29" s="134">
+        <f>E27-E28</f>
+        <v/>
+      </c>
+      <c r="F29" s="134">
+        <f>F27-F28</f>
+        <v/>
+      </c>
+      <c r="G29" s="134">
+        <f>G27-G28</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30" ht="19" customHeight="1">
+      <c r="B30" s="133" t="inlineStr">
+        <is>
+          <t>Resultado acumulado</t>
+        </is>
+      </c>
+      <c r="C30" s="135">
+        <f>C29</f>
+        <v/>
+      </c>
+      <c r="D30" s="135">
+        <f>C30+D29</f>
+        <v/>
+      </c>
+      <c r="E30" s="135">
+        <f>D30+E29</f>
+        <v/>
+      </c>
+      <c r="F30" s="135">
+        <f>E30+F29</f>
+        <v/>
+      </c>
+      <c r="G30" s="135">
+        <f>F30+G29</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32" ht="8" customHeight="1"/>
+    <row r="33" ht="24" customHeight="1">
+      <c r="B33" s="139" t="inlineStr">
+        <is>
+          <t>P&amp;L · TARGET MODELO P&amp;L  (700 usuarios Año 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="B34" s="116" t="inlineStr"/>
+      <c r="C34" s="117" t="inlineStr">
+        <is>
+          <t>Año 1</t>
+        </is>
+      </c>
+      <c r="D34" s="117" t="inlineStr">
+        <is>
+          <t>Año 2</t>
+        </is>
+      </c>
+      <c r="E34" s="117" t="inlineStr">
+        <is>
+          <t>Año 3</t>
+        </is>
+      </c>
+      <c r="F34" s="117" t="inlineStr">
+        <is>
+          <t>Año 4</t>
+        </is>
+      </c>
+      <c r="G34" s="117" t="inlineStr">
+        <is>
+          <t>Año 5</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="19" customHeight="1">
+      <c r="B35" s="118" t="inlineStr">
+        <is>
+          <t>Nuevos usuarios captados</t>
+        </is>
+      </c>
+      <c r="C35" s="96" t="n">
+        <v>700</v>
+      </c>
+      <c r="D35" s="140">
+        <f>C35+100</f>
+        <v/>
+      </c>
+      <c r="E35" s="140">
+        <f>D35+300</f>
+        <v/>
+      </c>
+      <c r="F35" s="140">
+        <f>E35+400</f>
+        <v/>
+      </c>
+      <c r="G35" s="140">
+        <f>F35+350</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36" ht="19" customHeight="1">
+      <c r="B36" s="118" t="inlineStr">
+        <is>
+          <t>Usuarios activos fin de año</t>
+        </is>
+      </c>
+      <c r="C36" s="140">
+        <f>C35</f>
+        <v/>
+      </c>
+      <c r="D36" s="140">
+        <f>ROUND(C35*0.75+D35,0)</f>
+        <v/>
+      </c>
+      <c r="E36" s="140">
+        <f>ROUND(D35*0.75+E35,0)</f>
+        <v/>
+      </c>
+      <c r="F36" s="140">
+        <f>ROUND(E35*0.75+F35,0)</f>
+        <v/>
+      </c>
+      <c r="G36" s="140">
+        <f>ROUND(F35*0.75+G35,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37" ht="19" customHeight="1">
+      <c r="B37" s="118" t="inlineStr">
+        <is>
+          <t>Ingresos (usuarios × 83€)</t>
+        </is>
+      </c>
+      <c r="C37" s="141">
+        <f>C36*83</f>
+        <v/>
+      </c>
+      <c r="D37" s="141">
+        <f>D36*83</f>
+        <v/>
+      </c>
+      <c r="E37" s="141">
+        <f>E36*83</f>
+        <v/>
+      </c>
+      <c r="F37" s="141">
+        <f>F36*83</f>
+        <v/>
+      </c>
+      <c r="G37" s="141">
+        <f>G36*83</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38" ht="19" customHeight="1">
+      <c r="B38" s="118" t="inlineStr">
+        <is>
+          <t>Costes totales</t>
+        </is>
+      </c>
+      <c r="C38" s="132" t="n">
+        <v>120000</v>
+      </c>
+      <c r="D38" s="132" t="n">
+        <v>129000</v>
+      </c>
+      <c r="E38" s="132" t="n">
+        <v>155000</v>
+      </c>
+      <c r="F38" s="132" t="n">
+        <v>175000</v>
+      </c>
+      <c r="G38" s="132" t="n">
+        <v>185000</v>
+      </c>
+    </row>
+    <row r="39" ht="19" customHeight="1">
+      <c r="B39" s="133" t="inlineStr">
+        <is>
+          <t>Resultado anual</t>
+        </is>
+      </c>
+      <c r="C39" s="134">
+        <f>C37-C38</f>
+        <v/>
+      </c>
+      <c r="D39" s="134">
+        <f>D37-D38</f>
+        <v/>
+      </c>
+      <c r="E39" s="134">
+        <f>E37-E38</f>
+        <v/>
+      </c>
+      <c r="F39" s="134">
+        <f>F37-F38</f>
+        <v/>
+      </c>
+      <c r="G39" s="134">
+        <f>G37-G38</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40" ht="19" customHeight="1">
+      <c r="B40" s="133" t="inlineStr">
+        <is>
+          <t>Resultado acumulado</t>
+        </is>
+      </c>
+      <c r="C40" s="135">
+        <f>C39</f>
+        <v/>
+      </c>
+      <c r="D40" s="135">
+        <f>C40+D39</f>
+        <v/>
+      </c>
+      <c r="E40" s="135">
+        <f>D40+E39</f>
+        <v/>
+      </c>
+      <c r="F40" s="135">
+        <f>E40+F39</f>
+        <v/>
+      </c>
+      <c r="G40" s="135">
+        <f>F40+G39</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42" ht="8" customHeight="1"/>
+    <row r="43" ht="28" customHeight="1">
+      <c r="B43" s="142" t="inlineStr">
+        <is>
+          <t>RESUMEN — ¿CUÁNDO SE ALCANZA EL BREAK-EVEN?</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="B44" s="143" t="inlineStr">
+        <is>
+          <t>Escenario</t>
+        </is>
+      </c>
+      <c r="C44" s="144" t="inlineStr">
+        <is>
+          <t>Usuarios Y1</t>
+        </is>
+      </c>
+      <c r="D44" s="144" t="inlineStr">
+        <is>
+          <t>Break-even anual</t>
+        </is>
+      </c>
+      <c r="E44" s="144" t="inlineStr">
+        <is>
+          <t>Break-even acumulado</t>
+        </is>
+      </c>
+      <c r="F44" s="144" t="inlineStr">
+        <is>
+          <t>Resultado Y5</t>
+        </is>
+      </c>
+      <c r="G44" s="144" t="inlineStr">
+        <is>
+          <t>Acumulado Y5</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="B45" s="145" t="inlineStr">
+        <is>
+          <t>Realista (195u · CAC ~83€)</t>
+        </is>
+      </c>
+      <c r="C45" s="146" t="inlineStr"/>
+      <c r="D45" s="147" t="inlineStr">
+        <is>
+          <t>Año 5→</t>
+        </is>
+      </c>
+      <c r="E45" s="146" t="inlineStr">
+        <is>
+          <t>No en 5 años</t>
+        </is>
+      </c>
+      <c r="F45" s="146" t="inlineStr"/>
+      <c r="G45" s="146" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="B46" s="148" t="inlineStr">
+        <is>
+          <t>Optimista (515u · CAC ~40€)</t>
+        </is>
+      </c>
+      <c r="C46" s="149" t="inlineStr"/>
+      <c r="D46" s="150" t="inlineStr">
+        <is>
+          <t>Año 4</t>
+        </is>
+      </c>
+      <c r="E46" s="149" t="inlineStr">
+        <is>
+          <t>Final Año 4–5</t>
+        </is>
+      </c>
+      <c r="F46" s="149" t="inlineStr"/>
+      <c r="G46" s="149" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="B47" s="151" t="inlineStr">
+        <is>
+          <t>Target modelo (700u)</t>
+        </is>
+      </c>
+      <c r="C47" s="152" t="inlineStr"/>
+      <c r="D47" s="153" t="inlineStr">
+        <is>
+          <t>Año 3</t>
+        </is>
+      </c>
+      <c r="E47" s="152" t="inlineStr">
+        <is>
+          <t>Final Año 4</t>
+        </is>
+      </c>
+      <c r="F47" s="152" t="inlineStr"/>
+      <c r="G47" s="152" t="inlineStr"/>
+    </row>
+    <row r="49" ht="26" customHeight="1">
+      <c r="B49" s="115" t="inlineStr">
+        <is>
+          <t>SENSIBILIDAD — Presupuesto de marketing vs Usuarios captados Año 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="B50" s="116" t="inlineStr">
+        <is>
+          <t>Presupuesto marketing</t>
+        </is>
+      </c>
+      <c r="C50" s="154" t="inlineStr">
+        <is>
+          <t>30.000€</t>
+        </is>
+      </c>
+      <c r="D50" s="154" t="inlineStr">
+        <is>
+          <t>40.000€
+(actual)</t>
+        </is>
+      </c>
+      <c r="E50" s="154" t="inlineStr">
+        <is>
+          <t>50.000€</t>
+        </is>
+      </c>
+      <c r="F50" s="154" t="inlineStr">
+        <is>
+          <t>60.000€</t>
+        </is>
+      </c>
+      <c r="G50" s="154" t="inlineStr">
+        <is>
+          <t>75.000€</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="B51" s="118" t="inlineStr">
+        <is>
+          <t>Usuarios (CAC realista ~80€)</t>
+        </is>
+      </c>
+      <c r="C51" s="155" t="n">
+        <v>361</v>
+      </c>
+      <c r="D51" s="156" t="n">
+        <v>482</v>
+      </c>
+      <c r="E51" s="156" t="n">
+        <v>625</v>
+      </c>
+      <c r="F51" s="157" t="n">
+        <v>769</v>
+      </c>
+      <c r="G51" s="157" t="n">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="B52" s="118" t="inlineStr">
+        <is>
+          <t>Usuarios (CAC optimista ~25€)</t>
+        </is>
+      </c>
+      <c r="C52" s="157" t="n">
+        <v>857</v>
+      </c>
+      <c r="D52" s="157" t="n">
+        <v>1600</v>
+      </c>
+      <c r="E52" s="157" t="n">
+        <v>2273</v>
+      </c>
+      <c r="F52" s="157" t="n">
+        <v>3000</v>
+      </c>
+      <c r="G52" s="157" t="n">
+        <v>4167</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="B53" s="158" t="inlineStr">
+        <is>
+          <t>Budget mínimo para 700u realista</t>
+        </is>
+      </c>
+      <c r="C53" s="159" t="inlineStr">
+        <is>
+          <t>~58.100€  (700 × 83€)</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="B54" s="158" t="inlineStr">
+        <is>
+          <t>Budget mínimo para 700u optimista</t>
+        </is>
+      </c>
+      <c r="C54" s="159" t="inlineStr">
+        <is>
+          <t>~17.500€  (700 × 25€) → con mix 25%: total ~43.750€</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="26" customHeight="1">
+      <c r="B57" s="160" t="inlineStr">
+        <is>
+          <t>CONCLUSIONES Y RECOMENDACIONES</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="36" customHeight="1">
+      <c r="B58" s="161" t="inlineStr">
+        <is>
+          <t>⚠</t>
+        </is>
+      </c>
+      <c r="C58" s="162" t="inlineStr">
+        <is>
+          <t>REALISTA con 40k: break-even anual no se alcanza antes del Año 5. El acumulado sigue negativo en todo el horizonte de 5 años. Necesitas o más presupuesto o mejores conversiones.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="36" customHeight="1">
+      <c r="B59" s="163" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="C59" s="164" t="inlineStr">
+        <is>
+          <t>OPTIMISTA con 40k: break-even anual en Año 4. Acumulado positivo en Año 4–5. Manejable si los influencers y paid convierten bien desde el principio.</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="36" customHeight="1">
+      <c r="B60" s="165" t="inlineStr">
+        <is>
+          <t>★</t>
+        </is>
+      </c>
+      <c r="C60" s="166" t="inlineStr">
+        <is>
+          <t>TARGET 700u: requiere conversiones optimistas (CAC ~25€ en paid) con el presupuesto actual de 40k. Si el CAC sube a 40–50€, necesitas 48–55k para alcanzar 700u vía paid.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="36" customHeight="1">
+      <c r="B61" s="167" t="inlineStr">
+        <is>
+          <t>💡</t>
+        </is>
+      </c>
+      <c r="C61" s="168" t="inlineStr">
+        <is>
+          <t>PALANCA MÁS EFICIENTE: optimizar la tasa de conversión de landing page (de 4% → 8%) reduce el CAC a la mitad SIN aumentar presupuesto. Es la acción prioritaria en beta.</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" ht="36" customHeight="1">
+      <c r="B62" s="167" t="inlineStr">
+        <is>
+          <t>💡</t>
+        </is>
+      </c>
+      <c r="C62" s="168" t="inlineStr">
+        <is>
+          <t>ALTERNATIVA: mantener 40k pero redirigir más % a paid (35–40% en vez de 25%). Con 40k × 40% = 16k en paid / CAC 50€ = 320 usuarios solo de paid. Mejor que el mix actual en realista.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="16">
+    <mergeCell ref="B49:L49"/>
+    <mergeCell ref="A2:L2"/>
+    <mergeCell ref="B43:L43"/>
+    <mergeCell ref="C61:L61"/>
+    <mergeCell ref="C54:G54"/>
+    <mergeCell ref="B23:G23"/>
+    <mergeCell ref="A1:L1"/>
+    <mergeCell ref="B4:G4"/>
+    <mergeCell ref="C59:L59"/>
+    <mergeCell ref="C53:G53"/>
+    <mergeCell ref="B13:G13"/>
+    <mergeCell ref="C60:L60"/>
+    <mergeCell ref="C62:L62"/>
+    <mergeCell ref="C58:L58"/>
+    <mergeCell ref="B33:G33"/>
+    <mergeCell ref="B57:L57"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>